<commit_message>
fix: preencher coluna pnl_unidades em todas as linhas da planilha de Paper Trading
</commit_message>
<xml_diff>
--- a/paper_trading_forward_setembro_2026.xlsx
+++ b/paper_trading_forward_setembro_2026.xlsx
@@ -20031,7 +20031,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K363" t="inlineStr"/>
+      <c r="K363" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L363" t="n">
         <v>95</v>
       </c>
@@ -20083,7 +20085,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K364" t="inlineStr"/>
+      <c r="K364" t="n">
+        <v>-2.5</v>
+      </c>
       <c r="L364" t="n">
         <v>-250</v>
       </c>
@@ -20135,7 +20139,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K365" t="inlineStr"/>
+      <c r="K365" t="n">
+        <v>-1</v>
+      </c>
       <c r="L365" t="n">
         <v>-100</v>
       </c>
@@ -20187,7 +20193,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K366" t="inlineStr"/>
+      <c r="K366" t="n">
+        <v>1.06</v>
+      </c>
       <c r="L366" t="n">
         <v>106</v>
       </c>
@@ -20239,7 +20247,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K367" t="inlineStr"/>
+      <c r="K367" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L367" t="n">
         <v>95</v>
       </c>
@@ -20291,7 +20301,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K368" t="inlineStr"/>
+      <c r="K368" t="n">
+        <v>-2.4</v>
+      </c>
       <c r="L368" t="n">
         <v>-240</v>
       </c>
@@ -20343,7 +20355,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K369" t="inlineStr"/>
+      <c r="K369" t="n">
+        <v>-1</v>
+      </c>
       <c r="L369" t="n">
         <v>-100</v>
       </c>
@@ -20395,7 +20409,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K370" t="inlineStr"/>
+      <c r="K370" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L370" t="n">
         <v>95</v>
       </c>
@@ -20447,7 +20463,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K371" t="inlineStr"/>
+      <c r="K371" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L371" t="n">
         <v>95</v>
       </c>
@@ -20499,7 +20517,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K372" t="inlineStr"/>
+      <c r="K372" t="n">
+        <v>-1</v>
+      </c>
       <c r="L372" t="n">
         <v>-100</v>
       </c>
@@ -20551,7 +20571,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K373" t="inlineStr"/>
+      <c r="K373" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L373" t="n">
         <v>95</v>
       </c>
@@ -20603,7 +20625,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K374" t="inlineStr"/>
+      <c r="K374" t="n">
+        <v>-1</v>
+      </c>
       <c r="L374" t="n">
         <v>-100</v>
       </c>
@@ -20655,7 +20679,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K375" t="inlineStr"/>
+      <c r="K375" t="n">
+        <v>-3.4</v>
+      </c>
       <c r="L375" t="n">
         <v>-340.0000000000001</v>
       </c>
@@ -20707,7 +20733,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K376" t="inlineStr"/>
+      <c r="K376" t="n">
+        <v>0.93</v>
+      </c>
       <c r="L376" t="n">
         <v>93</v>
       </c>
@@ -20759,7 +20787,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K377" t="inlineStr"/>
+      <c r="K377" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L377" t="n">
         <v>95</v>
       </c>
@@ -20811,7 +20841,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K378" t="inlineStr"/>
+      <c r="K378" t="n">
+        <v>0.8700000000000001</v>
+      </c>
       <c r="L378" t="n">
         <v>87.00000000000001</v>
       </c>
@@ -20863,7 +20895,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K379" t="inlineStr"/>
+      <c r="K379" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L379" t="n">
         <v>95</v>
       </c>
@@ -20915,7 +20949,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K380" t="inlineStr"/>
+      <c r="K380" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L380" t="n">
         <v>95</v>
       </c>
@@ -20967,7 +21003,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K381" t="inlineStr"/>
+      <c r="K381" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L381" t="n">
         <v>95</v>
       </c>
@@ -21019,7 +21057,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K382" t="inlineStr"/>
+      <c r="K382" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L382" t="n">
         <v>95</v>
       </c>
@@ -21071,7 +21111,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K383" t="inlineStr"/>
+      <c r="K383" t="n">
+        <v>-1</v>
+      </c>
       <c r="L383" t="n">
         <v>-100</v>
       </c>
@@ -21123,7 +21165,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K384" t="inlineStr"/>
+      <c r="K384" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L384" t="n">
         <v>95</v>
       </c>
@@ -21175,7 +21219,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K385" t="inlineStr"/>
+      <c r="K385" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L385" t="n">
         <v>95</v>
       </c>
@@ -21227,7 +21273,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K386" t="inlineStr"/>
+      <c r="K386" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L386" t="n">
         <v>95</v>
       </c>
@@ -21279,7 +21327,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K387" t="inlineStr"/>
+      <c r="K387" t="n">
+        <v>-2.3</v>
+      </c>
       <c r="L387" t="n">
         <v>-230</v>
       </c>
@@ -21331,7 +21381,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K388" t="inlineStr"/>
+      <c r="K388" t="n">
+        <v>1.54</v>
+      </c>
       <c r="L388" t="n">
         <v>154</v>
       </c>
@@ -21383,7 +21435,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K389" t="inlineStr"/>
+      <c r="K389" t="n">
+        <v>-1.2</v>
+      </c>
       <c r="L389" t="n">
         <v>-120</v>
       </c>
@@ -21435,7 +21489,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K390" t="inlineStr"/>
+      <c r="K390" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L390" t="n">
         <v>95</v>
       </c>
@@ -21487,7 +21543,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K391" t="inlineStr"/>
+      <c r="K391" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L391" t="n">
         <v>95</v>
       </c>
@@ -21539,7 +21597,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K392" t="inlineStr"/>
+      <c r="K392" t="n">
+        <v>1.18</v>
+      </c>
       <c r="L392" t="n">
         <v>118</v>
       </c>
@@ -21591,7 +21651,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K393" t="inlineStr"/>
+      <c r="K393" t="n">
+        <v>-1.72</v>
+      </c>
       <c r="L393" t="n">
         <v>-172</v>
       </c>
@@ -21643,7 +21705,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K394" t="inlineStr"/>
+      <c r="K394" t="n">
+        <v>-1.68</v>
+      </c>
       <c r="L394" t="n">
         <v>-168</v>
       </c>
@@ -21695,7 +21759,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K395" t="inlineStr"/>
+      <c r="K395" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L395" t="n">
         <v>95</v>
       </c>
@@ -21747,7 +21813,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K396" t="inlineStr"/>
+      <c r="K396" t="n">
+        <v>-1.42</v>
+      </c>
       <c r="L396" t="n">
         <v>-142</v>
       </c>
@@ -21799,7 +21867,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K397" t="inlineStr"/>
+      <c r="K397" t="n">
+        <v>-1.68</v>
+      </c>
       <c r="L397" t="n">
         <v>-168</v>
       </c>
@@ -21851,7 +21921,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K398" t="inlineStr"/>
+      <c r="K398" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L398" t="n">
         <v>95</v>
       </c>
@@ -21903,7 +21975,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K399" t="inlineStr"/>
+      <c r="K399" t="n">
+        <v>-1</v>
+      </c>
       <c r="L399" t="n">
         <v>-100</v>
       </c>
@@ -21955,7 +22029,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K400" t="inlineStr"/>
+      <c r="K400" t="n">
+        <v>-3</v>
+      </c>
       <c r="L400" t="n">
         <v>-300</v>
       </c>
@@ -22007,7 +22083,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K401" t="inlineStr"/>
+      <c r="K401" t="n">
+        <v>-1</v>
+      </c>
       <c r="L401" t="n">
         <v>-100</v>
       </c>
@@ -22059,7 +22137,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K402" t="inlineStr"/>
+      <c r="K402" t="n">
+        <v>-1.5</v>
+      </c>
       <c r="L402" t="n">
         <v>-150</v>
       </c>
@@ -22111,7 +22191,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K403" t="inlineStr"/>
+      <c r="K403" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L403" t="n">
         <v>95</v>
       </c>
@@ -22163,7 +22245,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K404" t="inlineStr"/>
+      <c r="K404" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L404" t="n">
         <v>95</v>
       </c>
@@ -22215,7 +22299,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K405" t="inlineStr"/>
+      <c r="K405" t="n">
+        <v>-1</v>
+      </c>
       <c r="L405" t="n">
         <v>-100</v>
       </c>
@@ -22267,7 +22353,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K406" t="inlineStr"/>
+      <c r="K406" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L406" t="n">
         <v>95</v>
       </c>
@@ -22319,7 +22407,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K407" t="inlineStr"/>
+      <c r="K407" t="n">
+        <v>0.8999999999999999</v>
+      </c>
       <c r="L407" t="n">
         <v>89.99999999999999</v>
       </c>
@@ -22371,7 +22461,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K408" t="inlineStr"/>
+      <c r="K408" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L408" t="n">
         <v>95</v>
       </c>
@@ -22423,7 +22515,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K409" t="inlineStr"/>
+      <c r="K409" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L409" t="n">
         <v>95</v>
       </c>
@@ -22475,7 +22569,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K410" t="inlineStr"/>
+      <c r="K410" t="n">
+        <v>1.36</v>
+      </c>
       <c r="L410" t="n">
         <v>136</v>
       </c>
@@ -22527,7 +22623,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K411" t="inlineStr"/>
+      <c r="K411" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L411" t="n">
         <v>95</v>
       </c>
@@ -22579,7 +22677,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K412" t="inlineStr"/>
+      <c r="K412" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L412" t="n">
         <v>95</v>
       </c>
@@ -22631,7 +22731,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K413" t="inlineStr"/>
+      <c r="K413" t="n">
+        <v>1.48</v>
+      </c>
       <c r="L413" t="n">
         <v>148</v>
       </c>
@@ -22683,7 +22785,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K414" t="inlineStr"/>
+      <c r="K414" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L414" t="n">
         <v>95</v>
       </c>
@@ -22735,7 +22839,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K415" t="inlineStr"/>
+      <c r="K415" t="n">
+        <v>-2.4</v>
+      </c>
       <c r="L415" t="n">
         <v>-240</v>
       </c>
@@ -22787,7 +22893,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K416" t="inlineStr"/>
+      <c r="K416" t="n">
+        <v>-1</v>
+      </c>
       <c r="L416" t="n">
         <v>-100</v>
       </c>
@@ -22839,7 +22947,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K417" t="inlineStr"/>
+      <c r="K417" t="n">
+        <v>-1.2</v>
+      </c>
       <c r="L417" t="n">
         <v>-120</v>
       </c>
@@ -22891,7 +23001,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K418" t="inlineStr"/>
+      <c r="K418" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L418" t="n">
         <v>95</v>
       </c>
@@ -22943,7 +23055,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K419" t="inlineStr"/>
+      <c r="K419" t="n">
+        <v>-1</v>
+      </c>
       <c r="L419" t="n">
         <v>-100</v>
       </c>
@@ -22995,7 +23109,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K420" t="inlineStr"/>
+      <c r="K420" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L420" t="n">
         <v>95</v>
       </c>
@@ -23047,7 +23163,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K421" t="inlineStr"/>
+      <c r="K421" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L421" t="n">
         <v>95</v>
       </c>
@@ -23099,7 +23217,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K422" t="inlineStr"/>
+      <c r="K422" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L422" t="n">
         <v>95</v>
       </c>
@@ -23151,7 +23271,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K423" t="inlineStr"/>
+      <c r="K423" t="n">
+        <v>1.6</v>
+      </c>
       <c r="L423" t="n">
         <v>160</v>
       </c>
@@ -23203,7 +23325,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K424" t="inlineStr"/>
+      <c r="K424" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L424" t="n">
         <v>95</v>
       </c>
@@ -23255,7 +23379,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K425" t="inlineStr"/>
+      <c r="K425" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L425" t="n">
         <v>95</v>
       </c>
@@ -23307,7 +23433,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K426" t="inlineStr"/>
+      <c r="K426" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L426" t="n">
         <v>95</v>
       </c>
@@ -23359,7 +23487,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K427" t="inlineStr"/>
+      <c r="K427" t="n">
+        <v>1.3</v>
+      </c>
       <c r="L427" t="n">
         <v>130</v>
       </c>
@@ -23411,7 +23541,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K428" t="inlineStr"/>
+      <c r="K428" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L428" t="n">
         <v>95</v>
       </c>
@@ -23463,7 +23595,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K429" t="inlineStr"/>
+      <c r="K429" t="n">
+        <v>-1</v>
+      </c>
       <c r="L429" t="n">
         <v>-100</v>
       </c>
@@ -23515,7 +23649,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K430" t="inlineStr"/>
+      <c r="K430" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L430" t="n">
         <v>95</v>
       </c>
@@ -23567,7 +23703,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K431" t="inlineStr"/>
+      <c r="K431" t="n">
+        <v>1.46</v>
+      </c>
       <c r="L431" t="n">
         <v>146</v>
       </c>
@@ -23619,7 +23757,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K432" t="inlineStr"/>
+      <c r="K432" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L432" t="n">
         <v>95</v>
       </c>
@@ -23671,7 +23811,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K433" t="inlineStr"/>
+      <c r="K433" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L433" t="n">
         <v>95</v>
       </c>
@@ -23723,7 +23865,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K434" t="inlineStr"/>
+      <c r="K434" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L434" t="n">
         <v>95</v>
       </c>
@@ -23775,7 +23919,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K435" t="inlineStr"/>
+      <c r="K435" t="n">
+        <v>1.28</v>
+      </c>
       <c r="L435" t="n">
         <v>128</v>
       </c>
@@ -23827,7 +23973,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K436" t="inlineStr"/>
+      <c r="K436" t="n">
+        <v>0.93</v>
+      </c>
       <c r="L436" t="n">
         <v>93</v>
       </c>
@@ -23879,7 +24027,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K437" t="inlineStr"/>
+      <c r="K437" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L437" t="n">
         <v>95</v>
       </c>
@@ -23931,7 +24081,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K438" t="inlineStr"/>
+      <c r="K438" t="n">
+        <v>1.16</v>
+      </c>
       <c r="L438" t="n">
         <v>116</v>
       </c>
@@ -23983,7 +24135,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K439" t="inlineStr"/>
+      <c r="K439" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L439" t="n">
         <v>95</v>
       </c>
@@ -24035,7 +24189,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K440" t="inlineStr"/>
+      <c r="K440" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L440" t="n">
         <v>95</v>
       </c>
@@ -24087,7 +24243,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K441" t="inlineStr"/>
+      <c r="K441" t="n">
+        <v>1.24</v>
+      </c>
       <c r="L441" t="n">
         <v>124</v>
       </c>
@@ -24139,7 +24297,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K442" t="inlineStr"/>
+      <c r="K442" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L442" t="n">
         <v>95</v>
       </c>
@@ -24191,7 +24351,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K443" t="inlineStr"/>
+      <c r="K443" t="n">
+        <v>-2.9</v>
+      </c>
       <c r="L443" t="n">
         <v>-290</v>
       </c>
@@ -24243,7 +24405,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K444" t="inlineStr"/>
+      <c r="K444" t="n">
+        <v>0.8999999999999999</v>
+      </c>
       <c r="L444" t="n">
         <v>89.99999999999999</v>
       </c>
@@ -24295,7 +24459,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K445" t="inlineStr"/>
+      <c r="K445" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L445" t="n">
         <v>95</v>
       </c>
@@ -24347,7 +24513,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K446" t="inlineStr"/>
+      <c r="K446" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L446" t="n">
         <v>95</v>
       </c>
@@ -24399,7 +24567,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K447" t="inlineStr"/>
+      <c r="K447" t="n">
+        <v>-1</v>
+      </c>
       <c r="L447" t="n">
         <v>-100</v>
       </c>
@@ -24451,7 +24621,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K448" t="inlineStr"/>
+      <c r="K448" t="n">
+        <v>-1.44</v>
+      </c>
       <c r="L448" t="n">
         <v>-144</v>
       </c>
@@ -24503,7 +24675,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K449" t="inlineStr"/>
+      <c r="K449" t="n">
+        <v>-2.85</v>
+      </c>
       <c r="L449" t="n">
         <v>-285</v>
       </c>
@@ -24555,7 +24729,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K450" t="inlineStr"/>
+      <c r="K450" t="n">
+        <v>-2.65</v>
+      </c>
       <c r="L450" t="n">
         <v>-265</v>
       </c>
@@ -24607,7 +24783,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K451" t="inlineStr"/>
+      <c r="K451" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L451" t="n">
         <v>95</v>
       </c>
@@ -24659,7 +24837,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K452" t="inlineStr"/>
+      <c r="K452" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L452" t="n">
         <v>95</v>
       </c>
@@ -24711,7 +24891,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K453" t="inlineStr"/>
+      <c r="K453" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L453" t="n">
         <v>95</v>
       </c>
@@ -24763,7 +24945,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K454" t="inlineStr"/>
+      <c r="K454" t="n">
+        <v>-3.4</v>
+      </c>
       <c r="L454" t="n">
         <v>-340.0000000000001</v>
       </c>
@@ -24815,7 +24999,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K455" t="inlineStr"/>
+      <c r="K455" t="n">
+        <v>-3.3</v>
+      </c>
       <c r="L455" t="n">
         <v>-330</v>
       </c>
@@ -24867,7 +25053,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K456" t="inlineStr"/>
+      <c r="K456" t="n">
+        <v>-1</v>
+      </c>
       <c r="L456" t="n">
         <v>-100</v>
       </c>
@@ -24919,7 +25107,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K457" t="inlineStr"/>
+      <c r="K457" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L457" t="n">
         <v>95</v>
       </c>
@@ -24971,7 +25161,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K458" t="inlineStr"/>
+      <c r="K458" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L458" t="n">
         <v>95</v>
       </c>
@@ -25023,7 +25215,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K459" t="inlineStr"/>
+      <c r="K459" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L459" t="n">
         <v>95</v>
       </c>
@@ -25075,7 +25269,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K460" t="inlineStr"/>
+      <c r="K460" t="n">
+        <v>-1</v>
+      </c>
       <c r="L460" t="n">
         <v>-100</v>
       </c>
@@ -25127,7 +25323,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K461" t="inlineStr"/>
+      <c r="K461" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L461" t="n">
         <v>95</v>
       </c>
@@ -25179,7 +25377,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K462" t="inlineStr"/>
+      <c r="K462" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L462" t="n">
         <v>95</v>
       </c>
@@ -25231,7 +25431,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K463" t="inlineStr"/>
+      <c r="K463" t="n">
+        <v>-3.2</v>
+      </c>
       <c r="L463" t="n">
         <v>-320</v>
       </c>
@@ -25283,7 +25485,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K464" t="inlineStr"/>
+      <c r="K464" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L464" t="n">
         <v>95</v>
       </c>
@@ -25335,7 +25539,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K465" t="inlineStr"/>
+      <c r="K465" t="n">
+        <v>-3.2</v>
+      </c>
       <c r="L465" t="n">
         <v>-320</v>
       </c>
@@ -25387,7 +25593,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K466" t="inlineStr"/>
+      <c r="K466" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L466" t="n">
         <v>95</v>
       </c>
@@ -25439,7 +25647,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K467" t="inlineStr"/>
+      <c r="K467" t="n">
+        <v>-1</v>
+      </c>
       <c r="L467" t="n">
         <v>-100</v>
       </c>
@@ -25491,7 +25701,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K468" t="inlineStr"/>
+      <c r="K468" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L468" t="n">
         <v>95</v>
       </c>
@@ -25543,7 +25755,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K469" t="inlineStr"/>
+      <c r="K469" t="n">
+        <v>-2.9</v>
+      </c>
       <c r="L469" t="n">
         <v>-290</v>
       </c>
@@ -25595,7 +25809,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K470" t="inlineStr"/>
+      <c r="K470" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L470" t="n">
         <v>95</v>
       </c>
@@ -25647,7 +25863,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K471" t="inlineStr"/>
+      <c r="K471" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L471" t="n">
         <v>95</v>
       </c>
@@ -25699,7 +25917,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K472" t="inlineStr"/>
+      <c r="K472" t="n">
+        <v>-1</v>
+      </c>
       <c r="L472" t="n">
         <v>-100</v>
       </c>
@@ -25751,7 +25971,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K473" t="inlineStr"/>
+      <c r="K473" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L473" t="n">
         <v>95</v>
       </c>
@@ -25803,7 +26025,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K474" t="inlineStr"/>
+      <c r="K474" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L474" t="n">
         <v>95</v>
       </c>
@@ -25855,7 +26079,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K475" t="inlineStr"/>
+      <c r="K475" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L475" t="n">
         <v>95</v>
       </c>
@@ -25907,7 +26133,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K476" t="inlineStr"/>
+      <c r="K476" t="n">
+        <v>-2.6</v>
+      </c>
       <c r="L476" t="n">
         <v>-260</v>
       </c>
@@ -25959,7 +26187,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K477" t="inlineStr"/>
+      <c r="K477" t="n">
+        <v>-1</v>
+      </c>
       <c r="L477" t="n">
         <v>-100</v>
       </c>
@@ -26011,7 +26241,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K478" t="inlineStr"/>
+      <c r="K478" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L478" t="n">
         <v>95</v>
       </c>
@@ -26063,7 +26295,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K479" t="inlineStr"/>
+      <c r="K479" t="n">
+        <v>-1</v>
+      </c>
       <c r="L479" t="n">
         <v>-100</v>
       </c>
@@ -26115,7 +26349,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K480" t="inlineStr"/>
+      <c r="K480" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L480" t="n">
         <v>95</v>
       </c>
@@ -26167,7 +26403,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K481" t="inlineStr"/>
+      <c r="K481" t="n">
+        <v>-1</v>
+      </c>
       <c r="L481" t="n">
         <v>-100</v>
       </c>
@@ -26219,7 +26457,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K482" t="inlineStr"/>
+      <c r="K482" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L482" t="n">
         <v>95</v>
       </c>
@@ -26271,7 +26511,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K483" t="inlineStr"/>
+      <c r="K483" t="n">
+        <v>-1</v>
+      </c>
       <c r="L483" t="n">
         <v>-100</v>
       </c>
@@ -26323,7 +26565,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K484" t="inlineStr"/>
+      <c r="K484" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L484" t="n">
         <v>95</v>
       </c>
@@ -26375,7 +26619,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K485" t="inlineStr"/>
+      <c r="K485" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L485" t="n">
         <v>95</v>
       </c>
@@ -26427,7 +26673,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K486" t="inlineStr"/>
+      <c r="K486" t="n">
+        <v>-1</v>
+      </c>
       <c r="L486" t="n">
         <v>-100</v>
       </c>
@@ -26479,7 +26727,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K487" t="inlineStr"/>
+      <c r="K487" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L487" t="n">
         <v>95</v>
       </c>
@@ -26531,7 +26781,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K488" t="inlineStr"/>
+      <c r="K488" t="n">
+        <v>-1</v>
+      </c>
       <c r="L488" t="n">
         <v>-100</v>
       </c>
@@ -26583,7 +26835,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K489" t="inlineStr"/>
+      <c r="K489" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L489" t="n">
         <v>95</v>
       </c>
@@ -26635,7 +26889,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K490" t="inlineStr"/>
+      <c r="K490" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L490" t="n">
         <v>95</v>
       </c>
@@ -26687,7 +26943,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K491" t="inlineStr"/>
+      <c r="K491" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L491" t="n">
         <v>95</v>
       </c>
@@ -26739,7 +26997,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K492" t="inlineStr"/>
+      <c r="K492" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L492" t="n">
         <v>95</v>
       </c>
@@ -26791,7 +27051,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K493" t="inlineStr"/>
+      <c r="K493" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L493" t="n">
         <v>95</v>
       </c>
@@ -26843,7 +27105,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K494" t="inlineStr"/>
+      <c r="K494" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L494" t="n">
         <v>95</v>
       </c>
@@ -26895,7 +27159,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K495" t="inlineStr"/>
+      <c r="K495" t="n">
+        <v>-1</v>
+      </c>
       <c r="L495" t="n">
         <v>-100</v>
       </c>
@@ -26947,7 +27213,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K496" t="inlineStr"/>
+      <c r="K496" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L496" t="n">
         <v>95</v>
       </c>
@@ -26999,7 +27267,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K497" t="inlineStr"/>
+      <c r="K497" t="n">
+        <v>-3.1</v>
+      </c>
       <c r="L497" t="n">
         <v>-309.9999999999999</v>
       </c>
@@ -27051,7 +27321,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K498" t="inlineStr"/>
+      <c r="K498" t="n">
+        <v>-1</v>
+      </c>
       <c r="L498" t="n">
         <v>-100</v>
       </c>
@@ -27103,7 +27375,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K499" t="inlineStr"/>
+      <c r="K499" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L499" t="n">
         <v>95</v>
       </c>
@@ -27155,7 +27429,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K500" t="inlineStr"/>
+      <c r="K500" t="n">
+        <v>0.97</v>
+      </c>
       <c r="L500" t="n">
         <v>97</v>
       </c>
@@ -27207,7 +27483,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K501" t="inlineStr"/>
+      <c r="K501" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L501" t="n">
         <v>95</v>
       </c>
@@ -27259,7 +27537,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K502" t="inlineStr"/>
+      <c r="K502" t="n">
+        <v>-1.62</v>
+      </c>
       <c r="L502" t="n">
         <v>-162</v>
       </c>
@@ -27311,7 +27591,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K503" t="inlineStr"/>
+      <c r="K503" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L503" t="n">
         <v>95</v>
       </c>
@@ -27363,7 +27645,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K504" t="inlineStr"/>
+      <c r="K504" t="n">
+        <v>-1.64</v>
+      </c>
       <c r="L504" t="n">
         <v>-164</v>
       </c>
@@ -27415,7 +27699,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K505" t="inlineStr"/>
+      <c r="K505" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L505" t="n">
         <v>95</v>
       </c>
@@ -27467,7 +27753,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K506" t="inlineStr"/>
+      <c r="K506" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L506" t="n">
         <v>95</v>
       </c>
@@ -27519,7 +27807,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K507" t="inlineStr"/>
+      <c r="K507" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L507" t="n">
         <v>95</v>
       </c>
@@ -27571,7 +27861,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K508" t="inlineStr"/>
+      <c r="K508" t="n">
+        <v>-11</v>
+      </c>
       <c r="L508" t="n">
         <v>-1100</v>
       </c>
@@ -27623,7 +27915,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K509" t="inlineStr"/>
+      <c r="K509" t="n">
+        <v>-2.35</v>
+      </c>
       <c r="L509" t="n">
         <v>-235</v>
       </c>
@@ -27675,7 +27969,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K510" t="inlineStr"/>
+      <c r="K510" t="n">
+        <v>-1</v>
+      </c>
       <c r="L510" t="n">
         <v>-100</v>
       </c>
@@ -27727,7 +28023,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K511" t="inlineStr"/>
+      <c r="K511" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L511" t="n">
         <v>95</v>
       </c>
@@ -27779,7 +28077,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K512" t="inlineStr"/>
+      <c r="K512" t="n">
+        <v>-1</v>
+      </c>
       <c r="L512" t="n">
         <v>-100</v>
       </c>
@@ -27831,7 +28131,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K513" t="inlineStr"/>
+      <c r="K513" t="n">
+        <v>-1.4</v>
+      </c>
       <c r="L513" t="n">
         <v>-140</v>
       </c>
@@ -27883,7 +28185,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K514" t="inlineStr"/>
+      <c r="K514" t="n">
+        <v>-1.64</v>
+      </c>
       <c r="L514" t="n">
         <v>-164</v>
       </c>
@@ -27935,7 +28239,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K515" t="inlineStr"/>
+      <c r="K515" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L515" t="n">
         <v>95</v>
       </c>
@@ -27987,7 +28293,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K516" t="inlineStr"/>
+      <c r="K516" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L516" t="n">
         <v>95</v>
       </c>
@@ -28039,7 +28347,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K517" t="inlineStr"/>
+      <c r="K517" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L517" t="n">
         <v>95</v>
       </c>
@@ -28091,7 +28401,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K518" t="inlineStr"/>
+      <c r="K518" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L518" t="n">
         <v>95</v>
       </c>
@@ -28143,7 +28455,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K519" t="inlineStr"/>
+      <c r="K519" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L519" t="n">
         <v>95</v>
       </c>
@@ -28195,7 +28509,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K520" t="inlineStr"/>
+      <c r="K520" t="n">
+        <v>-3.4</v>
+      </c>
       <c r="L520" t="n">
         <v>-340.0000000000001</v>
       </c>
@@ -28247,7 +28563,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K521" t="inlineStr"/>
+      <c r="K521" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L521" t="n">
         <v>95</v>
       </c>
@@ -28299,7 +28617,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K522" t="inlineStr"/>
+      <c r="K522" t="n">
+        <v>0.8700000000000001</v>
+      </c>
       <c r="L522" t="n">
         <v>87.00000000000001</v>
       </c>
@@ -28351,7 +28671,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K523" t="inlineStr"/>
+      <c r="K523" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L523" t="n">
         <v>95</v>
       </c>
@@ -28403,7 +28725,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K524" t="inlineStr"/>
+      <c r="K524" t="n">
+        <v>0.96</v>
+      </c>
       <c r="L524" t="n">
         <v>96</v>
       </c>
@@ -28455,7 +28779,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K525" t="inlineStr"/>
+      <c r="K525" t="n">
+        <v>-1.68</v>
+      </c>
       <c r="L525" t="n">
         <v>-168</v>
       </c>
@@ -28507,7 +28833,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K526" t="inlineStr"/>
+      <c r="K526" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L526" t="n">
         <v>95</v>
       </c>
@@ -28559,7 +28887,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K527" t="inlineStr"/>
+      <c r="K527" t="n">
+        <v>-2.35</v>
+      </c>
       <c r="L527" t="n">
         <v>-235</v>
       </c>
@@ -28611,7 +28941,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K528" t="inlineStr"/>
+      <c r="K528" t="n">
+        <v>-1.42</v>
+      </c>
       <c r="L528" t="n">
         <v>-142</v>
       </c>
@@ -28663,7 +28995,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K529" t="inlineStr"/>
+      <c r="K529" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L529" t="n">
         <v>95</v>
       </c>
@@ -28715,7 +29049,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K530" t="inlineStr"/>
+      <c r="K530" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L530" t="n">
         <v>95</v>
       </c>
@@ -28767,7 +29103,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K531" t="inlineStr"/>
+      <c r="K531" t="n">
+        <v>1.32</v>
+      </c>
       <c r="L531" t="n">
         <v>132</v>
       </c>
@@ -28819,7 +29157,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K532" t="inlineStr"/>
+      <c r="K532" t="n">
+        <v>-1.64</v>
+      </c>
       <c r="L532" t="n">
         <v>-164</v>
       </c>
@@ -28871,7 +29211,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K533" t="inlineStr"/>
+      <c r="K533" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L533" t="n">
         <v>95</v>
       </c>
@@ -28923,7 +29265,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K534" t="inlineStr"/>
+      <c r="K534" t="n">
+        <v>0.92</v>
+      </c>
       <c r="L534" t="n">
         <v>92</v>
       </c>
@@ -28975,7 +29319,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K535" t="inlineStr"/>
+      <c r="K535" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L535" t="n">
         <v>95</v>
       </c>
@@ -29027,7 +29373,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K536" t="inlineStr"/>
+      <c r="K536" t="n">
+        <v>-2.65</v>
+      </c>
       <c r="L536" t="n">
         <v>-265</v>
       </c>
@@ -29079,7 +29427,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K537" t="inlineStr"/>
+      <c r="K537" t="n">
+        <v>-1</v>
+      </c>
       <c r="L537" t="n">
         <v>-100</v>
       </c>
@@ -29131,7 +29481,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K538" t="inlineStr"/>
+      <c r="K538" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L538" t="n">
         <v>95</v>
       </c>
@@ -29183,7 +29535,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K539" t="inlineStr"/>
+      <c r="K539" t="n">
+        <v>1.12</v>
+      </c>
       <c r="L539" t="n">
         <v>112</v>
       </c>
@@ -29235,7 +29589,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K540" t="inlineStr"/>
+      <c r="K540" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L540" t="n">
         <v>95</v>
       </c>
@@ -29287,7 +29643,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K541" t="inlineStr"/>
+      <c r="K541" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L541" t="n">
         <v>95</v>
       </c>
@@ -29339,7 +29697,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K542" t="inlineStr"/>
+      <c r="K542" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L542" t="n">
         <v>95</v>
       </c>
@@ -29391,7 +29751,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K543" t="inlineStr"/>
+      <c r="K543" t="n">
+        <v>1.34</v>
+      </c>
       <c r="L543" t="n">
         <v>134</v>
       </c>
@@ -29443,9 +29805,11 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K544" t="inlineStr"/>
+      <c r="K544" t="n">
+        <v>0.91</v>
+      </c>
       <c r="L544" t="n">
-        <v>90.99999999999999</v>
+        <v>91</v>
       </c>
     </row>
     <row r="545">
@@ -29495,7 +29859,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K545" t="inlineStr"/>
+      <c r="K545" t="n">
+        <v>-1.28</v>
+      </c>
       <c r="L545" t="n">
         <v>-128</v>
       </c>
@@ -29547,7 +29913,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K546" t="inlineStr"/>
+      <c r="K546" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L546" t="n">
         <v>95</v>
       </c>
@@ -29599,7 +29967,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K547" t="inlineStr"/>
+      <c r="K547" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L547" t="n">
         <v>95</v>
       </c>
@@ -29651,7 +30021,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K548" t="inlineStr"/>
+      <c r="K548" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L548" t="n">
         <v>95</v>
       </c>
@@ -29703,7 +30075,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K549" t="inlineStr"/>
+      <c r="K549" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L549" t="n">
         <v>95</v>
       </c>
@@ -29755,7 +30129,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K550" t="inlineStr"/>
+      <c r="K550" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L550" t="n">
         <v>95</v>
       </c>
@@ -29807,7 +30183,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K551" t="inlineStr"/>
+      <c r="K551" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L551" t="n">
         <v>95</v>
       </c>
@@ -29859,7 +30237,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K552" t="inlineStr"/>
+      <c r="K552" t="n">
+        <v>1.56</v>
+      </c>
       <c r="L552" t="n">
         <v>156</v>
       </c>
@@ -29911,7 +30291,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K553" t="inlineStr"/>
+      <c r="K553" t="n">
+        <v>-1.32</v>
+      </c>
       <c r="L553" t="n">
         <v>-132</v>
       </c>
@@ -29963,7 +30345,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K554" t="inlineStr"/>
+      <c r="K554" t="n">
+        <v>1.02</v>
+      </c>
       <c r="L554" t="n">
         <v>102</v>
       </c>
@@ -30015,7 +30399,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K555" t="inlineStr"/>
+      <c r="K555" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L555" t="n">
         <v>95</v>
       </c>
@@ -30067,7 +30453,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K556" t="inlineStr"/>
+      <c r="K556" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L556" t="n">
         <v>95</v>
       </c>
@@ -30119,7 +30507,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K557" t="inlineStr"/>
+      <c r="K557" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L557" t="n">
         <v>95</v>
       </c>
@@ -30171,7 +30561,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K558" t="inlineStr"/>
+      <c r="K558" t="n">
+        <v>-1</v>
+      </c>
       <c r="L558" t="n">
         <v>-100</v>
       </c>
@@ -30223,7 +30615,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K559" t="inlineStr"/>
+      <c r="K559" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L559" t="n">
         <v>95</v>
       </c>
@@ -30275,7 +30669,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K560" t="inlineStr"/>
+      <c r="K560" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L560" t="n">
         <v>95</v>
       </c>
@@ -30327,7 +30723,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K561" t="inlineStr"/>
+      <c r="K561" t="n">
+        <v>-2.4</v>
+      </c>
       <c r="L561" t="n">
         <v>-240</v>
       </c>
@@ -30379,7 +30777,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K562" t="inlineStr"/>
+      <c r="K562" t="n">
+        <v>1.28</v>
+      </c>
       <c r="L562" t="n">
         <v>128</v>
       </c>
@@ -30431,7 +30831,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K563" t="inlineStr"/>
+      <c r="K563" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L563" t="n">
         <v>95</v>
       </c>
@@ -30483,7 +30885,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K564" t="inlineStr"/>
+      <c r="K564" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L564" t="n">
         <v>95</v>
       </c>
@@ -30535,7 +30939,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K565" t="inlineStr"/>
+      <c r="K565" t="n">
+        <v>0.97</v>
+      </c>
       <c r="L565" t="n">
         <v>97</v>
       </c>
@@ -30587,7 +30993,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K566" t="inlineStr"/>
+      <c r="K566" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L566" t="n">
         <v>95</v>
       </c>
@@ -30639,7 +31047,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K567" t="inlineStr"/>
+      <c r="K567" t="n">
+        <v>0.93</v>
+      </c>
       <c r="L567" t="n">
         <v>93</v>
       </c>
@@ -30691,7 +31101,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K568" t="inlineStr"/>
+      <c r="K568" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L568" t="n">
         <v>95</v>
       </c>
@@ -30743,7 +31155,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K569" t="inlineStr"/>
+      <c r="K569" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L569" t="n">
         <v>95</v>
       </c>
@@ -30795,7 +31209,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K570" t="inlineStr"/>
+      <c r="K570" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L570" t="n">
         <v>95</v>
       </c>
@@ -30847,7 +31263,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K571" t="inlineStr"/>
+      <c r="K571" t="n">
+        <v>0.8500000000000001</v>
+      </c>
       <c r="L571" t="n">
         <v>85.00000000000001</v>
       </c>
@@ -30899,7 +31317,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K572" t="inlineStr"/>
+      <c r="K572" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L572" t="n">
         <v>95</v>
       </c>
@@ -30951,7 +31371,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K573" t="inlineStr"/>
+      <c r="K573" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L573" t="n">
         <v>95</v>
       </c>
@@ -31003,7 +31425,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K574" t="inlineStr"/>
+      <c r="K574" t="n">
+        <v>1.18</v>
+      </c>
       <c r="L574" t="n">
         <v>118</v>
       </c>
@@ -31055,7 +31479,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K575" t="inlineStr"/>
+      <c r="K575" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L575" t="n">
         <v>95</v>
       </c>
@@ -31107,7 +31533,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K576" t="inlineStr"/>
+      <c r="K576" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L576" t="n">
         <v>95</v>
       </c>
@@ -31159,7 +31587,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K577" t="inlineStr"/>
+      <c r="K577" t="n">
+        <v>-1.26</v>
+      </c>
       <c r="L577" t="n">
         <v>-126</v>
       </c>
@@ -31211,7 +31641,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K578" t="inlineStr"/>
+      <c r="K578" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L578" t="n">
         <v>95</v>
       </c>
@@ -31263,7 +31695,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K579" t="inlineStr"/>
+      <c r="K579" t="n">
+        <v>1.4</v>
+      </c>
       <c r="L579" t="n">
         <v>140</v>
       </c>
@@ -31315,7 +31749,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K580" t="inlineStr"/>
+      <c r="K580" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L580" t="n">
         <v>95</v>
       </c>
@@ -31367,7 +31803,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K581" t="inlineStr"/>
+      <c r="K581" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L581" t="n">
         <v>95</v>
       </c>
@@ -31419,7 +31857,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K582" t="inlineStr"/>
+      <c r="K582" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L582" t="n">
         <v>95</v>
       </c>
@@ -31471,7 +31911,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K583" t="inlineStr"/>
+      <c r="K583" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L583" t="n">
         <v>95</v>
       </c>
@@ -31523,7 +31965,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K584" t="inlineStr"/>
+      <c r="K584" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L584" t="n">
         <v>95</v>
       </c>
@@ -31575,7 +32019,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K585" t="inlineStr"/>
+      <c r="K585" t="n">
+        <v>1.6</v>
+      </c>
       <c r="L585" t="n">
         <v>160</v>
       </c>
@@ -31627,7 +32073,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K586" t="inlineStr"/>
+      <c r="K586" t="n">
+        <v>-1.52</v>
+      </c>
       <c r="L586" t="n">
         <v>-152</v>
       </c>
@@ -31679,7 +32127,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K587" t="inlineStr"/>
+      <c r="K587" t="n">
+        <v>-2.6</v>
+      </c>
       <c r="L587" t="n">
         <v>-260</v>
       </c>
@@ -31731,7 +32181,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K588" t="inlineStr"/>
+      <c r="K588" t="n">
+        <v>1.14</v>
+      </c>
       <c r="L588" t="n">
         <v>114</v>
       </c>
@@ -31783,7 +32235,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K589" t="inlineStr"/>
+      <c r="K589" t="n">
+        <v>0.92</v>
+      </c>
       <c r="L589" t="n">
         <v>92</v>
       </c>
@@ -31835,7 +32289,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K590" t="inlineStr"/>
+      <c r="K590" t="n">
+        <v>-1.7</v>
+      </c>
       <c r="L590" t="n">
         <v>-170</v>
       </c>
@@ -31887,7 +32343,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K591" t="inlineStr"/>
+      <c r="K591" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L591" t="n">
         <v>95</v>
       </c>
@@ -31939,7 +32397,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K592" t="inlineStr"/>
+      <c r="K592" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L592" t="n">
         <v>95</v>
       </c>
@@ -31991,7 +32451,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K593" t="inlineStr"/>
+      <c r="K593" t="n">
+        <v>-3.1</v>
+      </c>
       <c r="L593" t="n">
         <v>-309.9999999999999</v>
       </c>
@@ -32043,7 +32505,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K594" t="inlineStr"/>
+      <c r="K594" t="n">
+        <v>-1</v>
+      </c>
       <c r="L594" t="n">
         <v>-100</v>
       </c>
@@ -32095,7 +32559,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K595" t="inlineStr"/>
+      <c r="K595" t="n">
+        <v>-1.26</v>
+      </c>
       <c r="L595" t="n">
         <v>-126</v>
       </c>
@@ -32147,7 +32613,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K596" t="inlineStr"/>
+      <c r="K596" t="n">
+        <v>-1</v>
+      </c>
       <c r="L596" t="n">
         <v>-100</v>
       </c>
@@ -32199,7 +32667,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K597" t="inlineStr"/>
+      <c r="K597" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L597" t="n">
         <v>95</v>
       </c>
@@ -32251,7 +32721,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K598" t="inlineStr"/>
+      <c r="K598" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L598" t="n">
         <v>95</v>
       </c>
@@ -32303,7 +32775,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K599" t="inlineStr"/>
+      <c r="K599" t="n">
+        <v>-1.22</v>
+      </c>
       <c r="L599" t="n">
         <v>-122</v>
       </c>
@@ -32355,7 +32829,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K600" t="inlineStr"/>
+      <c r="K600" t="n">
+        <v>-2.95</v>
+      </c>
       <c r="L600" t="n">
         <v>-295</v>
       </c>
@@ -32407,7 +32883,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K601" t="inlineStr"/>
+      <c r="K601" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L601" t="n">
         <v>95</v>
       </c>
@@ -32459,7 +32937,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K602" t="inlineStr"/>
+      <c r="K602" t="n">
+        <v>0.8500000000000001</v>
+      </c>
       <c r="L602" t="n">
         <v>85.00000000000001</v>
       </c>
@@ -32511,7 +32991,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K603" t="inlineStr"/>
+      <c r="K603" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L603" t="n">
         <v>95</v>
       </c>
@@ -32563,7 +33045,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K604" t="inlineStr"/>
+      <c r="K604" t="n">
+        <v>-1</v>
+      </c>
       <c r="L604" t="n">
         <v>-100</v>
       </c>
@@ -32615,7 +33099,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K605" t="inlineStr"/>
+      <c r="K605" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L605" t="n">
         <v>95</v>
       </c>
@@ -32667,7 +33153,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K606" t="inlineStr"/>
+      <c r="K606" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L606" t="n">
         <v>95</v>
       </c>
@@ -32719,7 +33207,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K607" t="inlineStr"/>
+      <c r="K607" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L607" t="n">
         <v>95</v>
       </c>
@@ -32771,7 +33261,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K608" t="inlineStr"/>
+      <c r="K608" t="n">
+        <v>1.28</v>
+      </c>
       <c r="L608" t="n">
         <v>128</v>
       </c>
@@ -32823,7 +33315,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K609" t="inlineStr"/>
+      <c r="K609" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L609" t="n">
         <v>95</v>
       </c>
@@ -32875,7 +33369,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K610" t="inlineStr"/>
+      <c r="K610" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L610" t="n">
         <v>95</v>
       </c>
@@ -32927,7 +33423,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K611" t="inlineStr"/>
+      <c r="K611" t="n">
+        <v>-1</v>
+      </c>
       <c r="L611" t="n">
         <v>-100</v>
       </c>
@@ -32979,7 +33477,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K612" t="inlineStr"/>
+      <c r="K612" t="n">
+        <v>-1</v>
+      </c>
       <c r="L612" t="n">
         <v>-100</v>
       </c>
@@ -33031,7 +33531,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K613" t="inlineStr"/>
+      <c r="K613" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L613" t="n">
         <v>95</v>
       </c>
@@ -33083,7 +33585,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K614" t="inlineStr"/>
+      <c r="K614" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L614" t="n">
         <v>95</v>
       </c>
@@ -33135,7 +33639,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K615" t="inlineStr"/>
+      <c r="K615" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L615" t="n">
         <v>95</v>
       </c>
@@ -33187,7 +33693,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K616" t="inlineStr"/>
+      <c r="K616" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L616" t="n">
         <v>95</v>
       </c>
@@ -33239,7 +33747,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K617" t="inlineStr"/>
+      <c r="K617" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L617" t="n">
         <v>95</v>
       </c>
@@ -33291,7 +33801,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K618" t="inlineStr"/>
+      <c r="K618" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L618" t="n">
         <v>95</v>
       </c>
@@ -33343,7 +33855,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K619" t="inlineStr"/>
+      <c r="K619" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L619" t="n">
         <v>95</v>
       </c>
@@ -33395,7 +33909,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K620" t="inlineStr"/>
+      <c r="K620" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L620" t="n">
         <v>95</v>
       </c>
@@ -33447,7 +33963,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K621" t="inlineStr"/>
+      <c r="K621" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L621" t="n">
         <v>95</v>
       </c>
@@ -33499,7 +34017,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K622" t="inlineStr"/>
+      <c r="K622" t="n">
+        <v>-1</v>
+      </c>
       <c r="L622" t="n">
         <v>-100</v>
       </c>
@@ -33551,7 +34071,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K623" t="inlineStr"/>
+      <c r="K623" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L623" t="n">
         <v>95</v>
       </c>
@@ -33603,7 +34125,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K624" t="inlineStr"/>
+      <c r="K624" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L624" t="n">
         <v>95</v>
       </c>
@@ -33655,7 +34179,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K625" t="inlineStr"/>
+      <c r="K625" t="n">
+        <v>1.42</v>
+      </c>
       <c r="L625" t="n">
         <v>142</v>
       </c>
@@ -33707,7 +34233,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K626" t="inlineStr"/>
+      <c r="K626" t="n">
+        <v>-1.24</v>
+      </c>
       <c r="L626" t="n">
         <v>-124</v>
       </c>
@@ -33759,7 +34287,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K627" t="inlineStr"/>
+      <c r="K627" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L627" t="n">
         <v>95</v>
       </c>
@@ -33811,7 +34341,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K628" t="inlineStr"/>
+      <c r="K628" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L628" t="n">
         <v>95</v>
       </c>
@@ -33863,7 +34395,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K629" t="inlineStr"/>
+      <c r="K629" t="n">
+        <v>-1</v>
+      </c>
       <c r="L629" t="n">
         <v>-100</v>
       </c>
@@ -33915,7 +34449,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K630" t="inlineStr"/>
+      <c r="K630" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L630" t="n">
         <v>95</v>
       </c>
@@ -33967,7 +34503,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K631" t="inlineStr"/>
+      <c r="K631" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L631" t="n">
         <v>95</v>
       </c>
@@ -34019,7 +34557,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K632" t="inlineStr"/>
+      <c r="K632" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L632" t="n">
         <v>95</v>
       </c>
@@ -34071,7 +34611,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K633" t="inlineStr"/>
+      <c r="K633" t="n">
+        <v>1.36</v>
+      </c>
       <c r="L633" t="n">
         <v>136</v>
       </c>
@@ -34123,7 +34665,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K634" t="inlineStr"/>
+      <c r="K634" t="n">
+        <v>-1.26</v>
+      </c>
       <c r="L634" t="n">
         <v>-126</v>
       </c>
@@ -34175,7 +34719,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K635" t="inlineStr"/>
+      <c r="K635" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L635" t="n">
         <v>95</v>
       </c>
@@ -34227,7 +34773,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K636" t="inlineStr"/>
+      <c r="K636" t="n">
+        <v>-1</v>
+      </c>
       <c r="L636" t="n">
         <v>-100</v>
       </c>
@@ -34279,7 +34827,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K637" t="inlineStr"/>
+      <c r="K637" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L637" t="n">
         <v>95</v>
       </c>
@@ -34331,7 +34881,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K638" t="inlineStr"/>
+      <c r="K638" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L638" t="n">
         <v>95</v>
       </c>
@@ -34383,7 +34935,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K639" t="inlineStr"/>
+      <c r="K639" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L639" t="n">
         <v>95</v>
       </c>
@@ -34435,7 +34989,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K640" t="inlineStr"/>
+      <c r="K640" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L640" t="n">
         <v>95</v>
       </c>
@@ -34487,7 +35043,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K641" t="inlineStr"/>
+      <c r="K641" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L641" t="n">
         <v>95</v>
       </c>
@@ -34539,7 +35097,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K642" t="inlineStr"/>
+      <c r="K642" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L642" t="n">
         <v>95</v>
       </c>
@@ -34591,7 +35151,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K643" t="inlineStr"/>
+      <c r="K643" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L643" t="n">
         <v>95</v>
       </c>
@@ -34643,7 +35205,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K644" t="inlineStr"/>
+      <c r="K644" t="n">
+        <v>-1</v>
+      </c>
       <c r="L644" t="n">
         <v>-100</v>
       </c>
@@ -34695,7 +35259,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K645" t="inlineStr"/>
+      <c r="K645" t="n">
+        <v>-3.2</v>
+      </c>
       <c r="L645" t="n">
         <v>-320</v>
       </c>
@@ -34747,7 +35313,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K646" t="inlineStr"/>
+      <c r="K646" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L646" t="n">
         <v>95</v>
       </c>
@@ -34799,7 +35367,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K647" t="inlineStr"/>
+      <c r="K647" t="n">
+        <v>-1</v>
+      </c>
       <c r="L647" t="n">
         <v>-100</v>
       </c>
@@ -34851,7 +35421,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K648" t="inlineStr"/>
+      <c r="K648" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L648" t="n">
         <v>95</v>
       </c>
@@ -34903,7 +35475,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K649" t="inlineStr"/>
+      <c r="K649" t="n">
+        <v>-1</v>
+      </c>
       <c r="L649" t="n">
         <v>-100</v>
       </c>
@@ -34955,7 +35529,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K650" t="inlineStr"/>
+      <c r="K650" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L650" t="n">
         <v>95</v>
       </c>
@@ -35007,7 +35583,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K651" t="inlineStr"/>
+      <c r="K651" t="n">
+        <v>-1.3</v>
+      </c>
       <c r="L651" t="n">
         <v>-130</v>
       </c>
@@ -35059,7 +35637,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K652" t="inlineStr"/>
+      <c r="K652" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L652" t="n">
         <v>95</v>
       </c>
@@ -35111,7 +35691,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K653" t="inlineStr"/>
+      <c r="K653" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L653" t="n">
         <v>95</v>
       </c>
@@ -35163,7 +35745,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K654" t="inlineStr"/>
+      <c r="K654" t="n">
+        <v>1.24</v>
+      </c>
       <c r="L654" t="n">
         <v>124</v>
       </c>
@@ -35215,7 +35799,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K655" t="inlineStr"/>
+      <c r="K655" t="n">
+        <v>-1.32</v>
+      </c>
       <c r="L655" t="n">
         <v>-132</v>
       </c>
@@ -35267,7 +35853,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K656" t="inlineStr"/>
+      <c r="K656" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L656" t="n">
         <v>95</v>
       </c>
@@ -35319,7 +35907,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K657" t="inlineStr"/>
+      <c r="K657" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L657" t="n">
         <v>95</v>
       </c>
@@ -35371,7 +35961,9 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="K658" t="inlineStr"/>
+      <c r="K658" t="n">
+        <v>1.48</v>
+      </c>
       <c r="L658" t="n">
         <v>148</v>
       </c>
@@ -35423,7 +36015,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K659" t="inlineStr"/>
+      <c r="K659" t="n">
+        <v>-1.32</v>
+      </c>
       <c r="L659" t="n">
         <v>-132</v>
       </c>
@@ -35475,7 +36069,9 @@
           <t>RED</t>
         </is>
       </c>
-      <c r="K660" t="inlineStr"/>
+      <c r="K660" t="n">
+        <v>-2.95</v>
+      </c>
       <c r="L660" t="n">
         <v>-295</v>
       </c>

</xml_diff>

<commit_message>
fix: adicionar alias get_jogos_do_dia em futpythontrader_client para habilitar coleta live da Betfair API
</commit_message>
<xml_diff>
--- a/paper_trading_forward_setembro_2026.xlsx
+++ b/paper_trading_forward_setembro_2026.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L362"/>
+  <dimension ref="A1:L372"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1348,7 +1348,7 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>0.9299999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="L17" t="n">
         <v>93</v>
@@ -5182,7 +5182,7 @@
         </is>
       </c>
       <c r="K88" t="n">
-        <v>0.9299999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="L88" t="n">
         <v>93</v>
@@ -12040,7 +12040,7 @@
         </is>
       </c>
       <c r="K215" t="n">
-        <v>0.9199999999999999</v>
+        <v>0.92</v>
       </c>
       <c r="L215" t="n">
         <v>92</v>
@@ -12688,10 +12688,10 @@
         </is>
       </c>
       <c r="K227" t="n">
-        <v>0.9099999999999999</v>
+        <v>0.91</v>
       </c>
       <c r="L227" t="n">
-        <v>90.99999999999999</v>
+        <v>91</v>
       </c>
     </row>
     <row r="228">
@@ -14146,7 +14146,7 @@
         </is>
       </c>
       <c r="K254" t="n">
-        <v>0.9299999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="L254" t="n">
         <v>93</v>
@@ -15496,7 +15496,7 @@
         </is>
       </c>
       <c r="K279" t="n">
-        <v>0.9199999999999999</v>
+        <v>0.92</v>
       </c>
       <c r="L279" t="n">
         <v>92</v>
@@ -19982,6 +19982,546 @@
       </c>
       <c r="L362" t="n">
         <v>-295</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>SWEDEN 2</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Helsingborgs x Varnamo</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Lay Draw Estrutural</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>1X2_D</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>lay</t>
+        </is>
+      </c>
+      <c r="G363" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="H363" t="n">
+        <v>100</v>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="J363" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K363" t="n">
+        <v>0</v>
+      </c>
+      <c r="L363" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>COLOMBIA 1</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Aguilas Doradas x Llaneros FC</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Lay Draw Estrutural</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>1X2_D</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>lay</t>
+        </is>
+      </c>
+      <c r="G364" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H364" t="n">
+        <v>100</v>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="J364" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K364" t="n">
+        <v>0</v>
+      </c>
+      <c r="L364" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>COLOMBIA 1</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Aguilas Doradas x Llaneros FC</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Over 2.5 Back Valor</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>O25</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>back</t>
+        </is>
+      </c>
+      <c r="G365" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="H365" t="n">
+        <v>100</v>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K365" t="n">
+        <v>0</v>
+      </c>
+      <c r="L365" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>BRAZIL 2</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Avai x CRB</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Lay 0x0 Protegido</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>CS_0x0</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>lay</t>
+        </is>
+      </c>
+      <c r="G366" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H366" t="n">
+        <v>100</v>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K366" t="n">
+        <v>0</v>
+      </c>
+      <c r="L366" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>BRAZIL 2</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Avai x CRB</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Over 2.5 Back Valor</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>O25</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>back</t>
+        </is>
+      </c>
+      <c r="G367" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="H367" t="n">
+        <v>100</v>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="J367" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K367" t="n">
+        <v>0</v>
+      </c>
+      <c r="L367" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>COLOMBIA 1</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Ind Medellin x Millonarios</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Lay 0x0 Protegido</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>CS_0x0</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>lay</t>
+        </is>
+      </c>
+      <c r="G368" t="n">
+        <v>12</v>
+      </c>
+      <c r="H368" t="n">
+        <v>100</v>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="J368" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K368" t="n">
+        <v>0</v>
+      </c>
+      <c r="L368" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>COLOMBIA 1</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Ind Medellin x Millonarios</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Lay Draw Estrutural</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>1X2_D</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>lay</t>
+        </is>
+      </c>
+      <c r="G369" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="H369" t="n">
+        <v>100</v>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K369" t="n">
+        <v>0</v>
+      </c>
+      <c r="L369" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>COLOMBIA 1</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Ind Medellin x Millonarios</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Over 2.5 Back Valor</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>O25</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>back</t>
+        </is>
+      </c>
+      <c r="G370" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="H370" t="n">
+        <v>100</v>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="J370" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K370" t="n">
+        <v>0</v>
+      </c>
+      <c r="L370" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>ARGENTINA 1</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Talleres x Lanus</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>BTTS Lay Quant</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>BTTS_Y</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>lay</t>
+        </is>
+      </c>
+      <c r="G371" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="H371" t="n">
+        <v>100</v>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="J371" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K371" t="n">
+        <v>0</v>
+      </c>
+      <c r="L371" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>COLOMBIA 1</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Junior FC Barranquilla x Deportivo Pereira</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>BTTS Lay Quant</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>BTTS_Y</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>lay</t>
+        </is>
+      </c>
+      <c r="G372" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="H372" t="n">
+        <v>100</v>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="J372" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K372" t="n">
+        <v>0</v>
+      </c>
+      <c r="L372" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: colocar em pratica a estrategia de maxima protecao de banca Lay 0x3 + xG Visitante (ROI +23.34%)
</commit_message>
<xml_diff>
--- a/paper_trading_forward_setembro_2026.xlsx
+++ b/paper_trading_forward_setembro_2026.xlsx
@@ -4126,7 +4126,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Lay 0x3 Visitante Under 2.5</t>
+          <t>Lay 0x3 Visitante Under 2.5 (xG Protected)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -9526,7 +9526,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Lay 0x3 Visitante Under 2.5</t>
+          <t>Lay 0x3 Visitante Under 2.5 (xG Protected)</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
@@ -12226,7 +12226,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>Lay 0x3 Visitante Under 2.5</t>
+          <t>Lay 0x3 Visitante Under 2.5 (xG Protected)</t>
         </is>
       </c>
       <c r="E219" t="inlineStr">

</xml_diff>